<commit_message>
new group-based vetting, admin IP allowlist, and email authentication features; updated documentation
</commit_message>
<xml_diff>
--- a/Sample_Dataset.xlsx
+++ b/Sample_Dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10901"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://zuac-my.sharepoint.com/personal/z9959_zu_ac_ae/Documents/ZU/MyTools/ConduVet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="246" documentId="11_C82EBED3F62F5C47A81CC0ADAF09D1234568C4E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF706C0A-588B-4D4C-A780-411532C7F4C8}"/>
+  <xr:revisionPtr revIDLastSave="266" documentId="11_C82EBED3F62F5C47A81CC0ADAF09D1234568C4E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79C6A372-B61E-4146-B554-D26AB531A925}"/>
   <bookViews>
-    <workbookView xWindow="9260" yWindow="11820" windowWidth="27640" windowHeight="9780" xr2:uid="{AB150B8C-8CCF-7443-9992-24B9B61CD0C2}"/>
+    <workbookView xWindow="9260" yWindow="7060" windowWidth="27640" windowHeight="14540" activeTab="1" xr2:uid="{AB150B8C-8CCF-7443-9992-24B9B61CD0C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="80">
   <si>
     <t>Year</t>
   </si>
@@ -276,6 +276,21 @@
   </si>
   <si>
     <t>Boolean</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>Group ID; Vetters can only see records of their assigned Group</t>
+  </si>
+  <si>
+    <t>zzz678</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Protected</t>
   </si>
 </sst>
 </file>
@@ -1075,7 +1090,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16106EC4-3BB4-DD42-9015-929FDC1FB953}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="18.6640625" style="33" customWidth="1"/>
@@ -1083,11 +1098,11 @@
     <col min="3" max="3" width="19.6640625" style="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.83203125" style="23" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.5" style="19" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5" style="18" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.83203125" style="6"/>
+    <col min="6" max="7" width="13.5" style="18" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.83203125" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15">
+    <row r="1" spans="1:7" ht="15">
       <c r="A1" s="29" t="s">
         <v>6</v>
       </c>
@@ -1106,8 +1121,11 @@
       <c r="F1" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="15">
+      <c r="G1" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15">
       <c r="A2" s="30" t="s">
         <v>19</v>
       </c>
@@ -1124,238 +1142,281 @@
       <c r="F2" s="10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="15">
+      <c r="G2" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="30">
       <c r="A3" s="30" t="s">
-        <v>18</v>
+        <v>75</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>27</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="E3" s="9"/>
       <c r="F3" s="10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="15">
+      <c r="G3" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15">
       <c r="A4" s="30" t="s">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" s="21">
-        <v>2026</v>
+        <v>27</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>40</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="15">
+      <c r="G4" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15">
       <c r="A5" s="30" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>14</v>
+        <v>41</v>
+      </c>
+      <c r="D5" s="21">
+        <v>2026</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="15">
+      <c r="G5" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15">
       <c r="A6" s="30" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E6" s="9"/>
       <c r="F6" s="10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="314">
+      <c r="G6" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15">
       <c r="A7" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>31</v>
+        <v>2</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>16</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="E7" s="9"/>
       <c r="F7" s="10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="90">
+      <c r="G7" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="314">
       <c r="A8" s="30" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>49</v>
+        <v>54</v>
+      </c>
+      <c r="B8" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>31</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>5</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>72</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="10" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="60">
+      <c r="G8" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="90">
       <c r="A9" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="60">
+      <c r="A10" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B10" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C10" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="36" t="s">
+      <c r="D10" s="36" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="14"/>
-      <c r="F9" s="10" t="s">
+      <c r="E10" s="14"/>
+      <c r="F10" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="30">
-      <c r="A10" s="31" t="s">
+      <c r="G10" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="30">
+      <c r="A11" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B11" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C11" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D11" s="15" t="s">
         <v>35</v>
-      </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="30">
-      <c r="A11" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>36</v>
       </c>
       <c r="E11" s="16"/>
       <c r="F11" s="17" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="15">
-      <c r="A12" s="32" t="s">
-        <v>73</v>
+      <c r="G11" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="30">
+      <c r="A12" s="31" t="s">
+        <v>21</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="11" t="b">
-        <v>0</v>
+        <v>45</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>36</v>
       </c>
       <c r="E12" s="16"/>
       <c r="F12" s="17" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="45">
-      <c r="A13" s="31" t="s">
-        <v>22</v>
+      <c r="G12" s="17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15">
+      <c r="A13" s="32" t="s">
+        <v>73</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>38</v>
+        <v>43</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="11" t="b">
+        <v>0</v>
       </c>
       <c r="E13" s="16"/>
       <c r="F13" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="45">
+      <c r="A14" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="16"/>
+      <c r="F14" s="17" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="15">
-      <c r="B14" s="24"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="28"/>
+      <c r="G14" s="17" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15">
+      <c r="B15" s="24"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D9" r:id="rId1" xr:uid="{A8C0AA18-849F-4C4A-A21E-97CB7AE1420E}"/>
+    <hyperlink ref="D10" r:id="rId1" xr:uid="{A8C0AA18-849F-4C4A-A21E-97CB7AE1420E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003701CD0AA27D7E49B2EBD118B743C068" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="84adf66037c2e333f03cf0d6f2f5f5a5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f8c4534e-65bf-4e9b-a1f1-a352e3723734" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5fc83c9ee1c6d66abecc145708d93584" ns2:_="">
     <xsd:import namespace="f8c4534e-65bf-4e9b-a1f1-a352e3723734"/>
@@ -1517,31 +1578,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C141DD21-E081-4789-AEEA-FE9688CBD4B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A2F51DE0-19D3-4CA2-9C91-F30FECDCB8B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="f8c4534e-65bf-4e9b-a1f1-a352e3723734"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{236E80D6-6192-44DC-9EC0-2E66E766169B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1557,4 +1609,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A2F51DE0-19D3-4CA2-9C91-F30FECDCB8B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f8c4534e-65bf-4e9b-a1f1-a352e3723734"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C141DD21-E081-4789-AEEA-FE9688CBD4B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>